<commit_message>
complete test cases & new bugs reports
</commit_message>
<xml_diff>
--- a/QA/Test-Cases.xlsx.xlsx
+++ b/QA/Test-Cases.xlsx.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pro\source\repos\StudentManagement.API\QA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92117E07-CAD6-4DC4-9F10-0EED4E2C38DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5175898D-CE92-452B-8FE0-712FD1304AD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1060" yWindow="1060" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="81">
   <si>
     <t>ID</t>
   </si>
@@ -91,19 +91,204 @@
   </si>
   <si>
     <t>Teachers</t>
+  </si>
+  <si>
+    <t>TC-STU-002</t>
+  </si>
+  <si>
+    <t>Create Student</t>
+  </si>
+  <si>
+    <t>TC-STU-003</t>
+  </si>
+  <si>
+    <t>TC-STU-004</t>
+  </si>
+  <si>
+    <t>TC-STU-005</t>
+  </si>
+  <si>
+    <t>TC-STU-006</t>
+  </si>
+  <si>
+    <t>TC-TEA-007</t>
+  </si>
+  <si>
+    <t>TC-TEA-009</t>
+  </si>
+  <si>
+    <t>TC-TEA-010</t>
+  </si>
+  <si>
+    <t>TC-TEA-011</t>
+  </si>
+  <si>
+    <t>TC-TEA-012</t>
+  </si>
+  <si>
+    <t>TC-TEA-013</t>
+  </si>
+  <si>
+    <t>TC-COU-014</t>
+  </si>
+  <si>
+    <t>TC-COU-015</t>
+  </si>
+  <si>
+    <t>TC-COU-016</t>
+  </si>
+  <si>
+    <t>Courses</t>
+  </si>
+  <si>
+    <t>verify student by id</t>
+  </si>
+  <si>
+    <t>modify student</t>
+  </si>
+  <si>
+    <t>delete student</t>
+  </si>
+  <si>
+    <t>add two students with same StudentNumber</t>
+  </si>
+  <si>
+    <t>create teacher</t>
+  </si>
+  <si>
+    <t>list of teachers</t>
+  </si>
+  <si>
+    <t>delete teacher</t>
+  </si>
+  <si>
+    <t>modify teacher</t>
+  </si>
+  <si>
+    <t>verify teacher by id</t>
+  </si>
+  <si>
+    <t>GET teacher by code</t>
+  </si>
+  <si>
+    <t>add teacher with incorrect format email</t>
+  </si>
+  <si>
+    <t>Add course</t>
+  </si>
+  <si>
+    <t>list of courses</t>
+  </si>
+  <si>
+    <t>modify course</t>
+  </si>
+  <si>
+    <t>API running,teachers exist</t>
+  </si>
+  <si>
+    <t>API running,courses exist</t>
+  </si>
+  <si>
+    <t>TC-STU-017</t>
+  </si>
+  <si>
+    <t>Get student by invalid ID</t>
+  </si>
+  <si>
+    <t>ID=20</t>
+  </si>
+  <si>
+    <t>Valid student JSON</t>
+  </si>
+  <si>
+    <t>Valid teacher JSON</t>
+  </si>
+  <si>
+    <t>Valid course JSON</t>
+  </si>
+  <si>
+    <t>Email=abc</t>
+  </si>
+  <si>
+    <t>StudentNumber=ST89012</t>
+  </si>
+  <si>
+    <t>GET /api/teachers</t>
+  </si>
+  <si>
+    <t>TeacherCode=AB2345</t>
+  </si>
+  <si>
+    <t>GET /api/Courses</t>
+  </si>
+  <si>
+    <t>404 Not Found</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>ID=5</t>
+  </si>
+  <si>
+    <t>200 OK + JSON OBJECT</t>
+  </si>
+  <si>
+    <t>201 created</t>
+  </si>
+  <si>
+    <t>201 Created + JSON object</t>
+  </si>
+  <si>
+    <t>API running,student exist</t>
+  </si>
+  <si>
+    <t>ID=1 , valid student JSON</t>
+  </si>
+  <si>
+    <t>204No Content</t>
+  </si>
+  <si>
+    <t>204 No Content</t>
+  </si>
+  <si>
+    <t>ID=7</t>
+  </si>
+  <si>
+    <t>400 Bad Request</t>
+  </si>
+  <si>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API running,Database </t>
+  </si>
+  <si>
+    <t>500Internal Server Error</t>
+  </si>
+  <si>
+    <t>ID=3</t>
+  </si>
+  <si>
+    <t>ID=2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -126,8 +311,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -408,15 +596,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.81640625" customWidth="1"/>
     <col min="2" max="2" width="13.36328125" customWidth="1"/>
-    <col min="3" max="3" width="15.08984375" customWidth="1"/>
-    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="3" max="3" width="38.6328125" customWidth="1"/>
+    <col min="4" max="5" width="24.08984375" customWidth="1"/>
     <col min="6" max="6" width="23.7265625" customWidth="1"/>
-    <col min="7" max="7" width="19.08984375" customWidth="1"/>
+    <col min="7" max="7" width="23.1796875" customWidth="1"/>
     <col min="8" max="8" width="23.08984375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -484,12 +672,516 @@
         <v>18</v>
       </c>
     </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" t="s">
+        <v>77</v>
+      </c>
+      <c r="G3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H3" t="s">
+        <v>68</v>
+      </c>
+      <c r="I3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G4" t="s">
+        <v>66</v>
+      </c>
+      <c r="H4" t="s">
+        <v>67</v>
+      </c>
+      <c r="I4" t="s">
+        <v>65</v>
+      </c>
+      <c r="J4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>70</v>
+      </c>
+      <c r="G5" t="s">
+        <v>71</v>
+      </c>
+      <c r="H5" t="s">
+        <v>73</v>
+      </c>
+      <c r="I5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" t="s">
+        <v>73</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>70</v>
+      </c>
+      <c r="G6" t="s">
+        <v>74</v>
+      </c>
+      <c r="H6" t="s">
+        <v>72</v>
+      </c>
+      <c r="I6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F7" t="s">
+        <v>77</v>
+      </c>
+      <c r="G7" t="s">
+        <v>60</v>
+      </c>
+      <c r="H7" t="s">
+        <v>68</v>
+      </c>
+      <c r="I7" t="s">
+        <v>18</v>
+      </c>
+      <c r="J7" t="s">
+        <v>18</v>
+      </c>
+    </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="B8" t="s">
         <v>20</v>
+      </c>
+      <c r="C8" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" t="s">
+        <v>69</v>
+      </c>
+      <c r="E8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" t="s">
+        <v>77</v>
+      </c>
+      <c r="G8" t="s">
+        <v>57</v>
+      </c>
+      <c r="H8" t="s">
+        <v>69</v>
+      </c>
+      <c r="I8" t="s">
+        <v>18</v>
+      </c>
+      <c r="J8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" t="s">
+        <v>76</v>
+      </c>
+      <c r="F9" t="s">
+        <v>51</v>
+      </c>
+      <c r="G9" t="s">
+        <v>61</v>
+      </c>
+      <c r="H9" t="s">
+        <v>78</v>
+      </c>
+      <c r="I9" t="s">
+        <v>18</v>
+      </c>
+      <c r="J9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" t="s">
+        <v>43</v>
+      </c>
+      <c r="D10" t="s">
+        <v>73</v>
+      </c>
+      <c r="E10" t="s">
+        <v>76</v>
+      </c>
+      <c r="F10" t="s">
+        <v>77</v>
+      </c>
+      <c r="G10" t="s">
+        <v>66</v>
+      </c>
+      <c r="H10" t="s">
+        <v>78</v>
+      </c>
+      <c r="I10" t="s">
+        <v>18</v>
+      </c>
+      <c r="J10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" t="s">
+        <v>73</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>77</v>
+      </c>
+      <c r="G11" t="s">
+        <v>66</v>
+      </c>
+      <c r="H11" t="s">
+        <v>73</v>
+      </c>
+      <c r="I11" t="s">
+        <v>18</v>
+      </c>
+      <c r="J11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" t="s">
+        <v>45</v>
+      </c>
+      <c r="D12" t="s">
+        <v>67</v>
+      </c>
+      <c r="E12" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" t="s">
+        <v>77</v>
+      </c>
+      <c r="G12" t="s">
+        <v>79</v>
+      </c>
+      <c r="H12" t="s">
+        <v>67</v>
+      </c>
+      <c r="I12" t="s">
+        <v>65</v>
+      </c>
+      <c r="J12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" t="s">
+        <v>46</v>
+      </c>
+      <c r="D13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>77</v>
+      </c>
+      <c r="G13" t="s">
+        <v>62</v>
+      </c>
+      <c r="H13" t="s">
+        <v>67</v>
+      </c>
+      <c r="I13" t="s">
+        <v>18</v>
+      </c>
+      <c r="J13" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" t="s">
+        <v>47</v>
+      </c>
+      <c r="D14" t="s">
+        <v>75</v>
+      </c>
+      <c r="E14" t="s">
+        <v>76</v>
+      </c>
+      <c r="F14" t="s">
+        <v>77</v>
+      </c>
+      <c r="G14" t="s">
+        <v>59</v>
+      </c>
+      <c r="H14" t="s">
+        <v>69</v>
+      </c>
+      <c r="I14" t="s">
+        <v>18</v>
+      </c>
+      <c r="J14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" t="s">
+        <v>69</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>77</v>
+      </c>
+      <c r="G15" t="s">
+        <v>58</v>
+      </c>
+      <c r="H15" t="s">
+        <v>69</v>
+      </c>
+      <c r="I15" t="s">
+        <v>18</v>
+      </c>
+      <c r="J15" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" t="s">
+        <v>49</v>
+      </c>
+      <c r="D16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E16" t="s">
+        <v>76</v>
+      </c>
+      <c r="F16" t="s">
+        <v>52</v>
+      </c>
+      <c r="G16" t="s">
+        <v>63</v>
+      </c>
+      <c r="H16" t="s">
+        <v>78</v>
+      </c>
+      <c r="I16" t="s">
+        <v>18</v>
+      </c>
+      <c r="J16" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" t="s">
+        <v>73</v>
+      </c>
+      <c r="E17" t="s">
+        <v>76</v>
+      </c>
+      <c r="F17" t="s">
+        <v>77</v>
+      </c>
+      <c r="G17" t="s">
+        <v>80</v>
+      </c>
+      <c r="H17" t="s">
+        <v>73</v>
+      </c>
+      <c r="I17" t="s">
+        <v>18</v>
+      </c>
+      <c r="J17" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>53</v>
+      </c>
+      <c r="B18" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" t="s">
+        <v>54</v>
+      </c>
+      <c r="D18" t="s">
+        <v>64</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>77</v>
+      </c>
+      <c r="G18" t="s">
+        <v>55</v>
+      </c>
+      <c r="H18" t="s">
+        <v>64</v>
+      </c>
+      <c r="I18" t="s">
+        <v>65</v>
+      </c>
+      <c r="J18" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>